<commit_message>
feat(samples): enrich datasets with cost, status, multi-year logistics series
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample_datasets/clientes_financieros_bi.xlsx
+++ b/sample_datasets/clientes_financieros_bi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,21 @@
           <t>Puntaje_Credito</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Plan_Activo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Fecha_Alta</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -493,6 +508,19 @@
       <c r="H2" t="n">
         <v>720</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -529,6 +557,19 @@
       <c r="H3" t="n">
         <v>810</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Básico</t>
+        </is>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2023-03-15</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -565,6 +606,19 @@
       <c r="H4" t="n">
         <v>690</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2023-06-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -601,6 +655,19 @@
       <c r="H5" t="n">
         <v>780</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2024-01-05</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +704,19 @@
       <c r="H6" t="n">
         <v>740</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Básico</t>
+        </is>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2024-02-18</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -673,6 +753,19 @@
       <c r="H7" t="n">
         <v>850</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2024-05-22</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -709,6 +802,19 @@
       <c r="H8" t="n">
         <v>650</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Básico</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2024-07-01</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -745,6 +851,19 @@
       <c r="H9" t="n">
         <v>790</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2024-08-14</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -781,6 +900,19 @@
       <c r="H10" t="n">
         <v>730</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2025-01-09</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -816,6 +948,19 @@
       </c>
       <c r="H11" t="n">
         <v>700</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Básico</t>
+        </is>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2025-03-12</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>